<commit_message>
2026-06-22 Added Daily Life Style Related Kanjis in Excel Data Source
</commit_message>
<xml_diff>
--- a/public/docs/kanji_n1.xlsx
+++ b/public/docs/kanji_n1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IG24-253\Documents\Work\ubuntu_practice\java\spring_boot\khans_kanji_english_practice\public\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ubuntu_practice\java\spring_boot\khans_kanji_english_practice\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F512A0-6F14-48D0-AF85-3FF232BB8E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="20" windowWidth="16100" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="138">
   <si>
     <t>Kanji</t>
   </si>
@@ -301,17 +302,188 @@
   <si>
     <t>n1_raise.jpg</t>
     <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>独立</t>
+  </si>
+  <si>
+    <t>忍耐</t>
+  </si>
+  <si>
+    <t>奉仕</t>
+  </si>
+  <si>
+    <t>自己改革</t>
+  </si>
+  <si>
+    <t>精神力</t>
+  </si>
+  <si>
+    <t>人生哲学</t>
+  </si>
+  <si>
+    <t>伝承</t>
+  </si>
+  <si>
+    <t>指導者</t>
+  </si>
+  <si>
+    <t>修行</t>
+  </si>
+  <si>
+    <t>洞察</t>
+  </si>
+  <si>
+    <t>鍛錬</t>
+  </si>
+  <si>
+    <t>知識</t>
+  </si>
+  <si>
+    <t>運命</t>
+  </si>
+  <si>
+    <t>覚醒</t>
+  </si>
+  <si>
+    <t>挑発</t>
+  </si>
+  <si>
+    <t>どくりつ</t>
+  </si>
+  <si>
+    <t>にんたい</t>
+  </si>
+  <si>
+    <t>ほうし</t>
+  </si>
+  <si>
+    <t>じこかいかく</t>
+  </si>
+  <si>
+    <t>せいしんりょく</t>
+  </si>
+  <si>
+    <t>じんせいてつがく</t>
+  </si>
+  <si>
+    <t>でんしょう</t>
+  </si>
+  <si>
+    <t>しどうしゃ</t>
+  </si>
+  <si>
+    <t>しゅぎょう</t>
+  </si>
+  <si>
+    <t>どうさつ</t>
+  </si>
+  <si>
+    <t>たんれん</t>
+  </si>
+  <si>
+    <t>ちしき</t>
+  </si>
+  <si>
+    <t>うんめい</t>
+  </si>
+  <si>
+    <t>かくせい</t>
+  </si>
+  <si>
+    <t>ちょうはつ</t>
+  </si>
+  <si>
+    <t>independence</t>
+  </si>
+  <si>
+    <t>patience</t>
+  </si>
+  <si>
+    <t>service</t>
+  </si>
+  <si>
+    <t>self-reform</t>
+  </si>
+  <si>
+    <t>mental strength</t>
+  </si>
+  <si>
+    <t>life philosophy</t>
+  </si>
+  <si>
+    <t>tradition/heritage</t>
+  </si>
+  <si>
+    <t>leader</t>
+  </si>
+  <si>
+    <t>training/discipline</t>
+  </si>
+  <si>
+    <t>insight</t>
+  </si>
+  <si>
+    <t>rigorous training</t>
+  </si>
+  <si>
+    <t>knowledge</t>
+  </si>
+  <si>
+    <t>fate/destiny</t>
+  </si>
+  <si>
+    <t>awakening</t>
+  </si>
+  <si>
+    <t>provocation/challenge</t>
+  </si>
+  <si>
+    <t>俳優</t>
+  </si>
+  <si>
+    <t>男優</t>
+  </si>
+  <si>
+    <t>女優</t>
+  </si>
+  <si>
+    <t>はいゆう</t>
+  </si>
+  <si>
+    <t>だんゆう</t>
+  </si>
+  <si>
+    <t>じょゆう</t>
+  </si>
+  <si>
+    <t>actor</t>
+  </si>
+  <si>
+    <t>male actor</t>
+  </si>
+  <si>
+    <t>actress</t>
+  </si>
+  <si>
+    <t>漫画</t>
+  </si>
+  <si>
+    <t>まんが</t>
+  </si>
+  <si>
+    <t>comics</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="ＭＳ Ｐゴシック"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -319,13 +491,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="ＭＳ Ｐゴシック"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="6"/>
-      <name val="ＭＳ Ｐゴシック"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -373,7 +545,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -389,9 +561,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -429,9 +601,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -466,7 +638,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -501,7 +673,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -674,11 +846,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,7 +864,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -706,7 +878,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -720,7 +892,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -734,7 +906,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -748,7 +920,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>49</v>
       </c>
@@ -762,7 +934,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>51</v>
       </c>
@@ -776,7 +948,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -790,7 +962,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>55</v>
       </c>
@@ -804,7 +976,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>57</v>
       </c>
@@ -818,7 +990,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>59</v>
       </c>
@@ -832,7 +1004,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>61</v>
       </c>
@@ -846,7 +1018,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>63</v>
       </c>
@@ -860,7 +1032,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -874,7 +1046,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -888,7 +1060,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>69</v>
       </c>
@@ -902,7 +1074,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>71</v>
       </c>
@@ -916,7 +1088,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -930,7 +1102,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>75</v>
       </c>
@@ -944,7 +1116,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>77</v>
       </c>
@@ -958,7 +1130,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>79</v>
       </c>
@@ -970,6 +1142,215 @@
       </c>
       <c r="D21" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" t="s">
+        <v>96</v>
+      </c>
+      <c r="C22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28" t="s">
+        <v>102</v>
+      </c>
+      <c r="C28" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" t="s">
+        <v>104</v>
+      </c>
+      <c r="C30" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" t="s">
+        <v>91</v>
+      </c>
+      <c r="B32" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33" t="s">
+        <v>107</v>
+      </c>
+      <c r="C33" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>93</v>
+      </c>
+      <c r="B34" t="s">
+        <v>108</v>
+      </c>
+      <c r="C34" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>94</v>
+      </c>
+      <c r="B35" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>95</v>
+      </c>
+      <c r="B36" t="s">
+        <v>110</v>
+      </c>
+      <c r="C36" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>126</v>
+      </c>
+      <c r="B37" t="s">
+        <v>129</v>
+      </c>
+      <c r="C37" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>128</v>
+      </c>
+      <c r="B39" t="s">
+        <v>131</v>
+      </c>
+      <c r="C39" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>135</v>
+      </c>
+      <c r="B40" t="s">
+        <v>136</v>
+      </c>
+      <c r="C40" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-06-23 Added Kanjis from N2S file in Excel Data Source
</commit_message>
<xml_diff>
--- a/public/docs/kanji_n1.xlsx
+++ b/public/docs/kanji_n1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ubuntu_practice\java\spring_boot\khans_kanji_english_practice\public\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ubuntu_practice\java\spring_boot\khans_kanji_english_practice\public\docs\temp_kanjis_to_add\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F512A0-6F14-48D0-AF85-3FF232BB8E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9995945D-FA0B-483F-83E1-A23815AB3C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="153">
   <si>
     <t>Kanji</t>
   </si>
@@ -473,6 +473,51 @@
   </si>
   <si>
     <t>comics</t>
+  </si>
+  <si>
+    <t>睡眠</t>
+  </si>
+  <si>
+    <t>永久</t>
+  </si>
+  <si>
+    <t>著者</t>
+  </si>
+  <si>
+    <t>著す</t>
+  </si>
+  <si>
+    <t>著しい</t>
+  </si>
+  <si>
+    <t>すいみん</t>
+  </si>
+  <si>
+    <t>えいきゅう</t>
+  </si>
+  <si>
+    <t>ちょしゃ</t>
+  </si>
+  <si>
+    <t>あらわす</t>
+  </si>
+  <si>
+    <t>いちじるしい</t>
+  </si>
+  <si>
+    <t>sleep</t>
+  </si>
+  <si>
+    <t>eternity</t>
+  </si>
+  <si>
+    <t>author</t>
+  </si>
+  <si>
+    <t>write; publish</t>
+  </si>
+  <si>
+    <t>remarkable</t>
   </si>
 </sst>
 </file>
@@ -847,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1351,6 +1396,61 @@
       </c>
       <c r="C40" t="s">
         <v>137</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41" t="s">
+        <v>143</v>
+      </c>
+      <c r="C41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>139</v>
+      </c>
+      <c r="B42" t="s">
+        <v>144</v>
+      </c>
+      <c r="C42" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43" t="s">
+        <v>145</v>
+      </c>
+      <c r="C43" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>141</v>
+      </c>
+      <c r="B44" t="s">
+        <v>146</v>
+      </c>
+      <c r="C44" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-09-12 Modified Kanjis in excel data sources
</commit_message>
<xml_diff>
--- a/public/docs/kanji_n1.xlsx
+++ b/public/docs/kanji_n1.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R89adb7798ed54bb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R8da59090838b463e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -449,9 +449,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">author</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">著す</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">あらわす</x:t>
@@ -1311,25 +1308,25 @@
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" t="s">
+      <x:c r="A44" t="str">
+        <x:v>著</x:v>
+      </x:c>
+      <x:c r="B44" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="B44" t="s">
+      <x:c r="C44" t="s">
         <x:v>148</x:v>
-      </x:c>
-      <x:c r="C44" t="s">
-        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="B45" t="s">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="B45" t="s">
+      <x:c r="C45" t="s">
         <x:v>151</x:v>
-      </x:c>
-      <x:c r="C45" t="s">
-        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -1778,7 +1775,7 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="4" t="str">
-        <x:v>恵まれる</x:v>
+        <x:v>恵</x:v>
       </x:c>
       <x:c r="B83" s="4" t="str">
         <x:v>めぐまれる</x:v>
@@ -2078,7 +2075,7 @@
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="4" t="str">
-        <x:v>健やかな</x:v>
+        <x:v>健</x:v>
       </x:c>
       <x:c r="B108" s="4" t="str">
         <x:v>すこやかな</x:v>
@@ -2234,7 +2231,7 @@
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="4" t="str">
-        <x:v>結ぶ</x:v>
+        <x:v>結</x:v>
       </x:c>
       <x:c r="B121" s="4" t="str">
         <x:v>むすぶ</x:v>
@@ -2258,7 +2255,7 @@
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="4" t="str">
-        <x:v>異なる</x:v>
+        <x:v>異</x:v>
       </x:c>
       <x:c r="B123" s="4" t="str">
         <x:v>ことなる</x:v>
@@ -2294,7 +2291,7 @@
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="4" t="str">
-        <x:v>整う</x:v>
+        <x:v>整</x:v>
       </x:c>
       <x:c r="B126" s="4" t="str">
         <x:v>ととのう</x:v>
@@ -2318,7 +2315,7 @@
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="4" t="str">
-        <x:v>暖かい</x:v>
+        <x:v>暖</x:v>
       </x:c>
       <x:c r="B128" s="4" t="str">
         <x:v>あたたかい</x:v>
@@ -2354,7 +2351,7 @@
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="4" t="str">
-        <x:v>保つ</x:v>
+        <x:v>保</x:v>
       </x:c>
       <x:c r="B131" s="4" t="str">
         <x:v>たもつ</x:v>
@@ -2546,7 +2543,7 @@
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="4" t="str">
-        <x:v>救う</x:v>
+        <x:v>救</x:v>
       </x:c>
       <x:c r="B147" s="4" t="str">
         <x:v>すくう</x:v>

</xml_diff>